<commit_message>
change an entry in this file to test multi value format parsing.
</commit_message>
<xml_diff>
--- a/t/data/trial/upload_phenotyping_spreadsheet_repetitive_measurements.xlsx
+++ b/t/data/trial/upload_phenotyping_spreadsheet_repetitive_measurements.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
   <si>
     <t xml:space="preserve">observationunit_name</t>
   </si>
@@ -175,16 +175,13 @@
     <t xml:space="preserve">49,2025-04-01 11:53:00</t>
   </si>
   <si>
-    <t xml:space="preserve">23,2025-04-01 11:53:00</t>
+    <t xml:space="preserve">23,2025-04-01 11:53:00|24,2025-04-01 11:53:00</t>
   </si>
   <si>
     <t xml:space="preserve">test_trial215</t>
   </si>
   <si>
     <t xml:space="preserve">50,2025-04-01 11:53:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24,2025-04-01 11:53:00</t>
   </si>
 </sst>
 </file>
@@ -288,37 +285,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -458,7 +455,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.27"/>
@@ -707,9 +704,7 @@
       <c r="C18" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>54</v>
-      </c>
+      <c r="D18" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="true" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>